<commit_message>
fix(import): apply blog fallback defaults
</commit_message>
<xml_diff>
--- a/public/templates/blog-import-template.xlsx
+++ b/public/templates/blog-import-template.xlsx
@@ -441,10 +441,10 @@
         <v>SH or RED</v>
       </c>
       <c r="B2" t="str">
-        <v>Full blog title</v>
+        <v>Full blog title (required)</v>
       </c>
       <c r="C2" t="str">
-        <v>Full published blog URL</v>
+        <v>Published URL (optional: fallback by Site)</v>
       </c>
       <c r="D2" t="str">
         <v>Blog writer name</v>
@@ -453,13 +453,13 @@
         <v>Person who published</v>
       </c>
       <c r="F2" t="str">
-        <v>Google Doc / writing link</v>
+        <v>Optional: defaults to https://docs.google.com/</v>
       </c>
       <c r="G2" t="str">
         <v>Date shown on blog (YYYY-MM-DD)</v>
       </c>
       <c r="H2" t="str">
-        <v>Internal publish date (YYYY-MM-DD)</v>
+        <v>Optional: defaults to Display Publish Date</v>
       </c>
     </row>
     <row r="3">
@@ -549,7 +549,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H27"/>
   <cols>
     <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -586,7 +586,7 @@
         <v>Live URL</v>
       </c>
       <c r="B6" t="str">
-        <v>Full published URL (must start with https://)</v>
+        <v>Optional. If empty, fallback is set by Site (SH→https://www.sighthound.com/blog/, RED→https://www.redactor.com/blog/)</v>
       </c>
     </row>
     <row r="7">
@@ -610,7 +610,7 @@
         <v>Draft Doc Link</v>
       </c>
       <c r="B9" t="str">
-        <v>Link to Google Doc or writing document (optional, but must start with https:// if provided)</v>
+        <v>Optional. Defaults to https://docs.google.com/ when selected and left empty</v>
       </c>
     </row>
     <row r="10">
@@ -626,7 +626,7 @@
         <v>Actual Publish Date</v>
       </c>
       <c r="B11" t="str">
-        <v>Internal publish date in YYYY-MM-DD format</v>
+        <v>Optional. Defaults to Display Publish Date when selected and left empty</v>
       </c>
     </row>
     <row r="13">
@@ -641,12 +641,12 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>• Duplicate blogs are detected using the Live URL</v>
+        <v>• Duplicate blogs are detected using the Live URL (canonical match)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>• Existing blogs with the same Live URL will be updated</v>
+        <v>• Existing blogs with the same Live URL are overwritten/updated with imported values</v>
       </c>
     </row>
     <row r="17">
@@ -656,58 +656,73 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>• All date fields must use YYYY-MM-DD format</v>
+        <v>• Missing Live URL uses Site fallback base URL</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>• Writer and Publisher names are case-insensitive</v>
+        <v>• Missing selected Draft Doc Link defaults to https://docs.google.com/</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>• New writer/publisher accounts will be auto-created if they don't exist</v>
+        <v>• Missing selected Actual Publish Date defaults to Display Publish Date</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>• All date fields must use YYYY-MM-DD format</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Example:</v>
+        <v>• Writer and Publisher names are case-insensitive</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
+        <v>• New writer/publisher accounts will be auto-created if they don't exist</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Example:</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
         <v>For a Sighthound blog about vehicle recognition:</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="str">
+    <row r="27">
+      <c r="A27" t="str">
         <v>SH</v>
       </c>
-      <c r="B24" t="str">
+      <c r="B27" t="str">
         <v>Vehicle Recognition for Parking Enforcement</v>
       </c>
-      <c r="C24" t="str">
+      <c r="C27" t="str">
         <v>https://www.sighthound.com/blog/vehicle-recognition-parking-enforcement</v>
       </c>
-      <c r="D24" t="str">
+      <c r="D27" t="str">
         <v>John Smith</v>
       </c>
-      <c r="E24" t="str">
+      <c r="E27" t="str">
         <v>Jane Doe</v>
       </c>
-      <c r="F24" t="str">
+      <c r="F27" t="str">
         <v>https://docs.google.com/document/d/abc123</v>
       </c>
-      <c r="G24" t="str">
+      <c r="G27" t="str">
         <v>2024-05-21</v>
       </c>
-      <c r="H24" t="str">
+      <c r="H27" t="str">
         <v>2024-05-20</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>